<commit_message>
feat: duplicatas e cline
</commit_message>
<xml_diff>
--- a/Excel/modelos/teste.xlsx
+++ b/Excel/modelos/teste.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/317ae1d27021fa3f/Desktop/Projetos/Utils/Excel/modelos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{57385B9D-0A60-4BC9-8BEF-AD337830B6D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C9276B9-ECEF-4D96-97FD-016CA09EDA98}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="8_{57385B9D-0A60-4BC9-8BEF-AD337830B6D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D21FA24F-FE0E-47E2-8F44-0DBACA1E87CB}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{878B9A18-36CE-4C4E-8AAF-9314A726B0AA}"/>
   </bookViews>
@@ -57,9 +57,6 @@
     <t>teste@gmail.com</t>
   </si>
   <si>
-    <t>0123456790</t>
-  </si>
-  <si>
     <t>Maria</t>
   </si>
   <si>
@@ -72,12 +69,6 @@
     <t>teste2@gmail.com</t>
   </si>
   <si>
-    <t>1123456791</t>
-  </si>
-  <si>
-    <t>2123456792</t>
-  </si>
-  <si>
     <t>Categoria</t>
   </si>
   <si>
@@ -88,6 +79,15 @@
   </si>
   <si>
     <t>Preto</t>
+  </si>
+  <si>
+    <t>21234567921</t>
+  </si>
+  <si>
+    <t>11234567911</t>
+  </si>
+  <si>
+    <t>01234567901</t>
   </si>
 </sst>
 </file>
@@ -159,9 +159,6 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -170,6 +167,9 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -195,15 +195,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{036D0A3E-37EC-42C0-BEAF-1D1678CBCFDB}" name="Tabela1" displayName="Tabela1" ref="A1:F4" totalsRowShown="0" headerRowDxfId="7" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{036D0A3E-37EC-42C0-BEAF-1D1678CBCFDB}" name="Tabela1" displayName="Tabela1" ref="A1:F4" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
   <autoFilter ref="A1:F4" xr:uid="{036D0A3E-37EC-42C0-BEAF-1D1678CBCFDB}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{50B4C9F6-BB35-4081-8C06-15B750F54536}" name="Nome" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{1436D997-97A4-4379-97F3-0D1A5B560B7B}" name="Email" dataDxfId="5" dataCellStyle="Hiperlink"/>
-    <tableColumn id="3" xr3:uid="{6999FFD4-842B-4512-8EAB-0D5AE08C8027}" name="CPF" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{D43919E5-6AA2-4227-8E9E-BA0262DBEAC0}" name="Telefone" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{EA36AE8C-BEEC-4A9D-9533-8429457F8465}" name="Dt_Nascimento" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{E5A37E91-DA87-4FA1-BA57-E9BD50A2A5DD}" name="Categoria" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{50B4C9F6-BB35-4081-8C06-15B750F54536}" name="Nome" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{1436D997-97A4-4379-97F3-0D1A5B560B7B}" name="Email" dataDxfId="4" dataCellStyle="Hiperlink"/>
+    <tableColumn id="3" xr3:uid="{6999FFD4-842B-4512-8EAB-0D5AE08C8027}" name="CPF" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{D43919E5-6AA2-4227-8E9E-BA0262DBEAC0}" name="Telefone" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{EA36AE8C-BEEC-4A9D-9533-8429457F8465}" name="Dt_Nascimento" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{E5A37E91-DA87-4FA1-BA57-E9BD50A2A5DD}" name="Categoria" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium22" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -534,7 +534,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -545,7 +545,7 @@
         <v>6</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="D2" s="2">
         <v>11912345678</v>
@@ -554,18 +554,18 @@
         <v>46119</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D3" s="2">
         <v>22912345678</v>
@@ -574,18 +574,18 @@
         <v>46246</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D4" s="2">
         <v>33912345678</v>
@@ -594,7 +594,7 @@
         <v>46052</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>